<commit_message>
feat(variant-4): add Ед. (шт.) column, rename Сегмент to Рейтинг with 6 colors & uncolored 5-col supplier order xlsx
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Заявки поставщикам (авторасчёт).xlsx
+++ b/Заявки поставщикам (авторасчёт).xlsx
@@ -193,7 +193,7 @@
       </c>
       <c r="L3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сегмент продаж</t>
+          <t xml:space="preserve">Рейтинг</t>
         </is>
       </c>
       <c r="M3" s="1" t="inlineStr">
@@ -233,7 +233,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H4" s="6">
@@ -290,7 +290,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H5" s="6">
@@ -347,7 +347,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H6" s="6">
@@ -404,7 +404,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H7" s="6">
@@ -461,7 +461,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H8" s="6">
@@ -518,7 +518,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H9" s="6">
@@ -575,7 +575,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H10" s="6">
@@ -632,7 +632,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H11" s="6">
@@ -689,7 +689,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H12" s="6">
@@ -746,7 +746,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H13" s="6">
@@ -803,7 +803,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H14" s="6">
@@ -860,7 +860,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H15" s="6">
@@ -917,7 +917,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H16" s="6">
@@ -974,7 +974,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H17" s="6">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H18" s="6">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H19" s="6">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H20" s="6">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H21" s="6">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H22" s="6">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H23" s="6">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H24" s="6">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H25" s="6">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H26" s="6">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H27" s="6">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H28" s="6">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H29" s="6">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H30" s="6">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H31" s="6">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H32" s="6">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H33" s="6">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H34" s="6">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H35" s="6">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H36" s="6">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H37" s="6">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H38" s="6">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H39" s="6">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H40" s="6">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H41" s="6">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H42" s="6">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H43" s="6">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H44" s="6">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H45" s="6">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H46" s="6">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H47" s="6">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H48" s="6">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H49" s="6">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H50" s="6">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H51" s="6">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H52" s="6">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H53" s="6">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведро</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H54" s="6">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H55" s="6">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H56" s="6">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H57" s="6">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H58" s="6">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H59" s="6">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H60" s="6">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H61" s="6">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H62" s="6">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H63" s="6">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H64" s="6">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H65" s="6">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H66" s="6">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H67" s="6">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H68" s="6">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H69" s="6">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведро</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H70" s="6">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H71" s="6">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H72" s="6">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H73" s="6">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведро</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H74" s="6">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H75" s="6">
@@ -4337,7 +4337,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H76" s="6">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведро</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H77" s="6">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведро</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H78" s="6">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведро</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H79" s="6">
@@ -4565,7 +4565,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведро</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H80" s="6">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведро</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H81" s="6">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H82" s="6">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H83" s="6">
@@ -4793,7 +4793,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H84" s="6">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H85" s="6">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H86" s="6">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H87" s="6">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H88" s="6">
@@ -5078,7 +5078,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H89" s="6">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H90" s="6">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H91" s="6">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H92" s="6">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H93" s="6">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">бут</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H94" s="6">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H95" s="6">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H96" s="6">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H97" s="6">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H98" s="6">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H99" s="6">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H100" s="6">
@@ -5762,7 +5762,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H101" s="6">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H102" s="6">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H103" s="6">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H104" s="6">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H105" s="6">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H106" s="6">
@@ -6104,7 +6104,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H107" s="6">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H108" s="6">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H109" s="6">
@@ -6275,7 +6275,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H110" s="6">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">бут</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H111" s="6">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">бут</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H112" s="6">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">бут</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H113" s="6">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H114" s="6">
@@ -6560,7 +6560,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H115" s="6">
@@ -6617,7 +6617,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H116" s="6">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H117" s="6">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H118" s="6">
@@ -6788,7 +6788,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H119" s="6">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H120" s="6">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H121" s="6">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H122" s="6">
@@ -7016,7 +7016,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H123" s="6">
@@ -7073,7 +7073,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H124" s="6">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H125" s="6">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H126" s="6">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H127" s="6">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H128" s="6">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H129" s="6">
@@ -7415,7 +7415,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H130" s="6">
@@ -7472,7 +7472,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H131" s="6">
@@ -7529,7 +7529,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H132" s="6">
@@ -7586,7 +7586,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H133" s="6">
@@ -7643,7 +7643,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H134" s="6">
@@ -7700,7 +7700,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H135" s="6">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H136" s="6">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H137" s="6">
@@ -7871,7 +7871,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H138" s="6">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H139" s="6">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H140" s="6">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H141" s="6">
@@ -8099,7 +8099,7 @@
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H142" s="6">
@@ -8156,7 +8156,7 @@
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H143" s="6">
@@ -8213,7 +8213,7 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H144" s="6">
@@ -8270,7 +8270,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H145" s="6">
@@ -8327,7 +8327,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H146" s="6">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H147" s="6">
@@ -8441,7 +8441,7 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H148" s="6">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H149" s="6">
@@ -8555,7 +8555,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H150" s="6">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H151" s="6">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H152" s="6">
@@ -8726,7 +8726,7 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H153" s="6">
@@ -8783,7 +8783,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H154" s="6">
@@ -8840,7 +8840,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H155" s="6">
@@ -8897,7 +8897,7 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H156" s="6">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H157" s="6">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H158" s="6">
@@ -9068,7 +9068,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H159" s="6">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H160" s="6">
@@ -9182,7 +9182,7 @@
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H161" s="6">
@@ -9239,7 +9239,7 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H162" s="6">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H163" s="6">
@@ -9353,7 +9353,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H164" s="6">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H165" s="6">
@@ -9467,7 +9467,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H166" s="6">
@@ -9524,7 +9524,7 @@
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H167" s="6">
@@ -9581,7 +9581,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">банка</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H168" s="6">
@@ -9638,7 +9638,7 @@
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H169" s="6">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H170" s="6">
@@ -9752,7 +9752,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H171" s="6">
@@ -9809,7 +9809,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H172" s="6">
@@ -9866,7 +9866,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H173" s="6">
@@ -9923,7 +9923,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H174" s="6">
@@ -9980,7 +9980,7 @@
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H175" s="6">
@@ -10037,7 +10037,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H176" s="6">
@@ -10094,7 +10094,7 @@
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H177" s="6">
@@ -10151,7 +10151,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H178" s="6">
@@ -10208,7 +10208,7 @@
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H179" s="6">
@@ -10265,7 +10265,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H180" s="6">
@@ -10322,7 +10322,7 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H181" s="6">
@@ -10379,7 +10379,7 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H182" s="6">
@@ -10436,7 +10436,7 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H183" s="6">
@@ -10493,7 +10493,7 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H184" s="6">
@@ -10550,7 +10550,7 @@
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H185" s="6">
@@ -10607,7 +10607,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H186" s="6">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H187" s="6">
@@ -10721,7 +10721,7 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H188" s="6">
@@ -10778,7 +10778,7 @@
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H189" s="6">
@@ -10835,7 +10835,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H190" s="6">
@@ -10892,7 +10892,7 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H191" s="6">
@@ -10949,7 +10949,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H192" s="6">
@@ -11006,7 +11006,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H193" s="6">
@@ -11063,7 +11063,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H194" s="6">
@@ -11120,7 +11120,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H195" s="6">
@@ -11177,7 +11177,7 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H196" s="6">
@@ -11234,7 +11234,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H197" s="6">
@@ -11291,7 +11291,7 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H198" s="6">
@@ -11348,7 +11348,7 @@
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H199" s="6">
@@ -11405,7 +11405,7 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H200" s="6">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H201" s="6">
@@ -11519,7 +11519,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H202" s="6">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H203" s="6">
@@ -11633,7 +11633,7 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H204" s="6">
@@ -11690,7 +11690,7 @@
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H205" s="6">
@@ -11747,7 +11747,7 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H206" s="6">
@@ -11804,7 +11804,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H207" s="6">
@@ -11861,7 +11861,7 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H208" s="6">
@@ -11918,7 +11918,7 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H209" s="6">
@@ -11975,7 +11975,7 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H210" s="6">
@@ -12032,7 +12032,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H211" s="6">
@@ -12089,7 +12089,7 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H212" s="6">
@@ -12146,7 +12146,7 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H213" s="6">
@@ -12203,7 +12203,7 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H214" s="6">
@@ -12260,7 +12260,7 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H215" s="6">
@@ -12317,7 +12317,7 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H216" s="6">
@@ -12374,7 +12374,7 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H217" s="6">
@@ -12431,7 +12431,7 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H218" s="6">
@@ -12488,7 +12488,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H219" s="6">
@@ -12545,7 +12545,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H220" s="6">
@@ -12602,7 +12602,7 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H221" s="6">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H222" s="6">
@@ -12716,7 +12716,7 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H223" s="6">
@@ -12773,7 +12773,7 @@
       </c>
       <c r="G224" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H224" s="6">
@@ -12830,7 +12830,7 @@
       </c>
       <c r="G225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H225" s="6">
@@ -12887,7 +12887,7 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H226" s="6">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H227" s="6">
@@ -13001,7 +13001,7 @@
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H228" s="6">
@@ -13058,7 +13058,7 @@
       </c>
       <c r="G229" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H229" s="6">
@@ -13115,7 +13115,7 @@
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H230" s="6">
@@ -13172,7 +13172,7 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H231" s="6">
@@ -13229,7 +13229,7 @@
       </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H232" s="6">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H233" s="6">
@@ -13343,7 +13343,7 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H234" s="6">
@@ -13400,7 +13400,7 @@
       </c>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H235" s="6">
@@ -13457,7 +13457,7 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H236" s="6">
@@ -13514,7 +13514,7 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H237" s="6">
@@ -13571,7 +13571,7 @@
       </c>
       <c r="G238" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H238" s="6">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H239" s="6">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H240" s="6">
@@ -13742,7 +13742,7 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H241" s="6">
@@ -13799,7 +13799,7 @@
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H242" s="6">
@@ -13856,7 +13856,7 @@
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H243" s="6">
@@ -13913,7 +13913,7 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H244" s="6">
@@ -13970,7 +13970,7 @@
       </c>
       <c r="G245" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H245" s="6">
@@ -14027,7 +14027,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H246" s="6">
@@ -14084,7 +14084,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H247" s="6">
@@ -14141,7 +14141,7 @@
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H248" s="6">
@@ -14198,7 +14198,7 @@
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H249" s="6">
@@ -14255,7 +14255,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H250" s="6">
@@ -14312,7 +14312,7 @@
       </c>
       <c r="G251" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H251" s="6">
@@ -14369,7 +14369,7 @@
       </c>
       <c r="G252" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H252" s="6">
@@ -14426,7 +14426,7 @@
       </c>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H253" s="6">
@@ -14483,7 +14483,7 @@
       </c>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H254" s="6">
@@ -14540,7 +14540,7 @@
       </c>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H255" s="6">
@@ -14597,7 +14597,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H256" s="6">
@@ -14654,7 +14654,7 @@
       </c>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H257" s="6">
@@ -14711,7 +14711,7 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H258" s="6">
@@ -14768,7 +14768,7 @@
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H259" s="6">
@@ -14825,7 +14825,7 @@
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H260" s="6">
@@ -14882,7 +14882,7 @@
       </c>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H261" s="6">
@@ -14939,7 +14939,7 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H262" s="6">
@@ -14996,7 +14996,7 @@
       </c>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H263" s="6">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H264" s="6">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H265" s="6">
@@ -15167,7 +15167,7 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H266" s="6">
@@ -15224,7 +15224,7 @@
       </c>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H267" s="6">
@@ -15281,7 +15281,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H268" s="6">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="G269" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H269" s="6">
@@ -15395,7 +15395,7 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H270" s="6">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H271" s="6">
@@ -15509,7 +15509,7 @@
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H272" s="6">
@@ -15566,7 +15566,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H273" s="6">
@@ -15623,7 +15623,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H274" s="6">
@@ -15680,7 +15680,7 @@
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H275" s="6">
@@ -15737,7 +15737,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H276" s="6">
@@ -15794,7 +15794,7 @@
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H277" s="6">
@@ -15851,7 +15851,7 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H278" s="6">
@@ -15908,7 +15908,7 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H279" s="6">
@@ -15965,7 +15965,7 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H280" s="6">
@@ -16022,7 +16022,7 @@
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H281" s="6">
@@ -16079,7 +16079,7 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H282" s="6">
@@ -16136,7 +16136,7 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H283" s="6">
@@ -16193,7 +16193,7 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H284" s="6">
@@ -16250,7 +16250,7 @@
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H285" s="6">
@@ -16307,7 +16307,7 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H286" s="6">
@@ -16364,7 +16364,7 @@
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H287" s="6">
@@ -16421,7 +16421,7 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H288" s="6">
@@ -16478,7 +16478,7 @@
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H289" s="6">
@@ -16535,7 +16535,7 @@
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H290" s="6">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H291" s="6">
@@ -16649,7 +16649,7 @@
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H292" s="6">
@@ -16706,7 +16706,7 @@
       </c>
       <c r="G293" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H293" s="6">
@@ -16763,7 +16763,7 @@
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H294" s="6">
@@ -16820,7 +16820,7 @@
       </c>
       <c r="G295" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H295" s="6">
@@ -16877,7 +16877,7 @@
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H296" s="6">
@@ -16934,7 +16934,7 @@
       </c>
       <c r="G297" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H297" s="6">
@@ -16991,7 +16991,7 @@
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H298" s="6">
@@ -17048,7 +17048,7 @@
       </c>
       <c r="G299" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H299" s="6">
@@ -17105,7 +17105,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H300" s="6">
@@ -17162,7 +17162,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H301" s="6">
@@ -17219,7 +17219,7 @@
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H302" s="6">
@@ -17276,7 +17276,7 @@
       </c>
       <c r="G303" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H303" s="6">
@@ -17333,7 +17333,7 @@
       </c>
       <c r="G304" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H304" s="6">
@@ -17390,7 +17390,7 @@
       </c>
       <c r="G305" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H305" s="6">
@@ -17447,7 +17447,7 @@
       </c>
       <c r="G306" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H306" s="6">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="G307" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H307" s="6">
@@ -17561,7 +17561,7 @@
       </c>
       <c r="G308" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H308" s="6">
@@ -17618,7 +17618,7 @@
       </c>
       <c r="G309" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H309" s="6">
@@ -17675,7 +17675,7 @@
       </c>
       <c r="G310" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H310" s="6">
@@ -17732,7 +17732,7 @@
       </c>
       <c r="G311" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H311" s="6">
@@ -17789,7 +17789,7 @@
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H312" s="6">
@@ -17846,7 +17846,7 @@
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H313" s="6">
@@ -17903,7 +17903,7 @@
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H314" s="6">
@@ -17960,7 +17960,7 @@
       </c>
       <c r="G315" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H315" s="6">
@@ -18017,7 +18017,7 @@
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H316" s="6">
@@ -18074,7 +18074,7 @@
       </c>
       <c r="G317" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H317" s="6">
@@ -18131,7 +18131,7 @@
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H318" s="6">
@@ -18188,7 +18188,7 @@
       </c>
       <c r="G319" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H319" s="6">
@@ -18245,7 +18245,7 @@
       </c>
       <c r="G320" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H320" s="6">
@@ -18302,7 +18302,7 @@
       </c>
       <c r="G321" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H321" s="6">
@@ -18359,7 +18359,7 @@
       </c>
       <c r="G322" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H322" s="6">
@@ -18416,7 +18416,7 @@
       </c>
       <c r="G323" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H323" s="6">
@@ -18473,7 +18473,7 @@
       </c>
       <c r="G324" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H324" s="6">
@@ -18530,7 +18530,7 @@
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H325" s="6">
@@ -18587,7 +18587,7 @@
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H326" s="6">
@@ -18644,7 +18644,7 @@
       </c>
       <c r="G327" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H327" s="6">
@@ -18701,7 +18701,7 @@
       </c>
       <c r="G328" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H328" s="6">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="G329" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H329" s="6">
@@ -18815,7 +18815,7 @@
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H330" s="6">
@@ -18872,7 +18872,7 @@
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H331" s="6">
@@ -18929,7 +18929,7 @@
       </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H332" s="6">
@@ -18986,7 +18986,7 @@
       </c>
       <c r="G333" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H333" s="6">
@@ -19043,7 +19043,7 @@
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H334" s="6">
@@ -19100,7 +19100,7 @@
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H335" s="6">
@@ -19157,7 +19157,7 @@
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H336" s="6">
@@ -19214,7 +19214,7 @@
       </c>
       <c r="G337" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H337" s="6">
@@ -19271,7 +19271,7 @@
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H338" s="6">
@@ -19328,7 +19328,7 @@
       </c>
       <c r="G339" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H339" s="6">
@@ -19385,7 +19385,7 @@
       </c>
       <c r="G340" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H340" s="6">
@@ -19442,7 +19442,7 @@
       </c>
       <c r="G341" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H341" s="6">
@@ -19499,7 +19499,7 @@
       </c>
       <c r="G342" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H342" s="6">
@@ -19556,7 +19556,7 @@
       </c>
       <c r="G343" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H343" s="6">
@@ -19613,7 +19613,7 @@
       </c>
       <c r="G344" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H344" s="6">
@@ -19670,7 +19670,7 @@
       </c>
       <c r="G345" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H345" s="6">
@@ -19727,7 +19727,7 @@
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H346" s="6">
@@ -19784,7 +19784,7 @@
       </c>
       <c r="G347" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H347" s="6">
@@ -19841,7 +19841,7 @@
       </c>
       <c r="G348" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H348" s="6">
@@ -19898,7 +19898,7 @@
       </c>
       <c r="G349" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H349" s="6">
@@ -19955,7 +19955,7 @@
       </c>
       <c r="G350" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H350" s="6">
@@ -20012,7 +20012,7 @@
       </c>
       <c r="G351" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H351" s="6">
@@ -20069,7 +20069,7 @@
       </c>
       <c r="G352" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H352" s="6">
@@ -20126,7 +20126,7 @@
       </c>
       <c r="G353" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H353" s="6">
@@ -20183,7 +20183,7 @@
       </c>
       <c r="G354" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H354" s="6">
@@ -20240,7 +20240,7 @@
       </c>
       <c r="G355" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H355" s="6">
@@ -20297,7 +20297,7 @@
       </c>
       <c r="G356" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H356" s="6">
@@ -20354,7 +20354,7 @@
       </c>
       <c r="G357" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H357" s="6">
@@ -20411,7 +20411,7 @@
       </c>
       <c r="G358" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H358" s="6">
@@ -20468,7 +20468,7 @@
       </c>
       <c r="G359" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H359" s="6">
@@ -20525,7 +20525,7 @@
       </c>
       <c r="G360" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H360" s="6">
@@ -20582,7 +20582,7 @@
       </c>
       <c r="G361" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H361" s="6">
@@ -20639,7 +20639,7 @@
       </c>
       <c r="G362" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">шт</t>
+          <t xml:space="preserve">шт.</t>
         </is>
       </c>
       <c r="H362" s="6">

</xml_diff>